<commit_message>
XRR developments and post transition to SQL improvements for XAS
+ reliability improvements to change_edge()
+ reliability improvements to all instances of linescans
+ make bmm_mongo connection for monitoring problem with streams
  getting lost on the way to SQL-backed tiled
+ make a tools that reports that problem on Slack when it happens
+ default ramp rate for lakeshore now 20
+ tile polling improvements in consumer plotting
+ grab and use entire data tables from Tiled in consumer
+ bad job of improving XRF and Mythen plots ... this needs fixing
+ harden file writing by polling better for records from tiled
+ make it possible to do xasxdi using mongo backend
+ templates and consumer tooling for XRR html reporting
</commit_message>
<xml_diff>
--- a/startup/lookup_table/Modes.xlsx
+++ b/startup/lookup_table/Modes.xlsx
@@ -11902,7 +11902,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ66"/>
-  <sheetFormatPr defaultColWidth="12.30859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.31640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.04"/>
@@ -15010,7 +15010,7 @@
         <v>189</v>
       </c>
       <c r="E56" s="60" t="n">
-        <v>121.584</v>
+        <v>118.322</v>
       </c>
       <c r="F56" s="25" t="n">
         <v>9251952</v>
@@ -15022,25 +15022,25 @@
         <v>4600216</v>
       </c>
       <c r="I56" s="60" t="n">
-        <v>55.662</v>
+        <v>52.4</v>
       </c>
       <c r="J56" s="23" t="n">
         <v>6151303</v>
       </c>
       <c r="K56" s="60" t="n">
-        <v>128.828</v>
+        <v>125.566</v>
       </c>
       <c r="L56" s="23" t="n">
         <v>9901395</v>
       </c>
       <c r="M56" s="60" t="n">
-        <v>129.115</v>
+        <v>125.853</v>
       </c>
       <c r="N56" s="23" t="n">
         <v>9901395</v>
       </c>
       <c r="O56" s="60" t="n">
-        <v>99.085</v>
+        <v>95.823</v>
       </c>
       <c r="P56" s="23" t="n">
         <v>8392750</v>
@@ -15126,7 +15126,7 @@
         <v>195</v>
       </c>
       <c r="E58" s="60" t="n">
-        <v>125.456</v>
+        <v>115.809</v>
       </c>
       <c r="F58" s="28" t="n">
         <v>5572330</v>
@@ -15138,25 +15138,25 @@
         <v>354340</v>
       </c>
       <c r="I58" s="60" t="n">
-        <v>51.435</v>
+        <v>41.788</v>
       </c>
       <c r="J58" s="32" t="n">
         <v>1952224</v>
       </c>
       <c r="K58" s="60" t="n">
-        <v>132.817</v>
+        <v>123.17</v>
       </c>
       <c r="L58" s="32" t="n">
         <v>6355689</v>
       </c>
       <c r="M58" s="60" t="n">
-        <v>132.859</v>
+        <v>123.212</v>
       </c>
       <c r="N58" s="32" t="n">
         <v>6355689</v>
       </c>
       <c r="O58" s="60" t="n">
-        <v>100.567</v>
+        <v>90.92</v>
       </c>
       <c r="P58" s="72" t="n">
         <v>4479629</v>
@@ -17226,7 +17226,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:K7"/>
-  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="33"/>
@@ -17405,7 +17405,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I36"/>
-  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="11.96"/>
@@ -17486,15 +17486,15 @@
       </c>
       <c r="E4" s="110" t="n">
         <f aca="false">'Modes A-F'!K56</f>
-        <v>128.828</v>
+        <v>125.566</v>
       </c>
       <c r="F4" s="110" t="n">
         <f aca="false">E4-B4*TAN(2*(F2-E2)/1000)</f>
-        <v>99.9169132666878</v>
+        <v>96.6549132666878</v>
       </c>
       <c r="G4" s="128" t="n">
         <f aca="false">'Modes A-F'!O56</f>
-        <v>99.085</v>
+        <v>95.823</v>
       </c>
       <c r="H4" s="129" t="n">
         <f aca="false">G4-F4</f>
@@ -17622,12 +17622,12 @@
       </c>
       <c r="E12" s="139" t="n">
         <f aca="false">'Modes A-F'!E58</f>
-        <v>125.456</v>
+        <v>115.809</v>
       </c>
       <c r="F12" s="139"/>
       <c r="G12" s="140" t="n">
         <f aca="false">E12-B12*TAN(2*(G9-E9)/1000)</f>
-        <v>127.995400033859</v>
+        <v>118.348400033859</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17757,7 +17757,7 @@
       </c>
       <c r="F23" s="144" t="n">
         <f aca="false">'Modes A-F'!I56</f>
-        <v>55.662</v>
+        <v>52.4</v>
       </c>
       <c r="G23" s="129" t="n">
         <f aca="false">E11-B23*TAN(2*(G19)/1000)+I17</f>
@@ -17779,7 +17779,7 @@
       </c>
       <c r="E24" s="139" t="n">
         <f aca="false">E12-B24*TAN(2*(E19)/1000)+I17</f>
-        <v>43.9748517843995</v>
+        <v>34.3278517843995</v>
       </c>
       <c r="F24" s="145" t="n">
         <f aca="false">'Modes A-F'!I57</f>
@@ -17787,7 +17787,7 @@
       </c>
       <c r="G24" s="146" t="n">
         <f aca="false">E12-B24*TAN(2*(G19)/1000)+I17</f>
-        <v>49.910766090482</v>
+        <v>40.263766090482</v>
       </c>
       <c r="H24" s="131"/>
       <c r="I24" s="147"/>
@@ -17941,7 +17941,7 @@
       </c>
       <c r="E36" s="139" t="n">
         <f aca="false">E12-B36*TAN(2*(E31)/1000)</f>
-        <v>11.596175674289</v>
+        <v>1.94917567428902</v>
       </c>
       <c r="F36" s="145" t="n">
         <f aca="false">'Modes A-F'!G57</f>
@@ -17949,7 +17949,7 @@
       </c>
       <c r="G36" s="139" t="n">
         <f aca="false">E12-B36*TAN(2*(G31)/1000)+I29</f>
-        <v>17.5324025227675</v>
+        <v>7.88540252276749</v>
       </c>
       <c r="H36" s="131"/>
       <c r="I36" s="147"/>
@@ -17976,7 +17976,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:CX484"/>
-  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="35.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="102" min="2" style="0" width="11.96"/>
@@ -24043,7 +24043,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G2383"/>
-  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.89453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="56.14"/>

</xml_diff>